<commit_message>
Second commit: added D=4 and E=5
</commit_message>
<xml_diff>
--- a/sampleexcel.xlsx
+++ b/sampleexcel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubProjects\MyThirdLocalRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D7B9540-3464-4550-9A7C-1092B6B7F476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C9895B-7BE8-4BF6-B204-4FC05E968C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{EF0871F4-5BC5-4CC6-BFB2-3372DD5EF46B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Alphabet</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -82,7 +88,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -105,16 +111,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -451,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9878FC8F-7A33-4FBD-B3F0-7B461849B564}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -490,6 +510,22 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Third commit: updated E from 5 to 50
</commit_message>
<xml_diff>
--- a/sampleexcel.xlsx
+++ b/sampleexcel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubProjects\MyThirdLocalRepo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C9895B-7BE8-4BF6-B204-4FC05E968C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049993AA-1655-49BA-92C1-84BB18C174C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{EF0871F4-5BC5-4CC6-BFB2-3372DD5EF46B}"/>
   </bookViews>
@@ -523,7 +523,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="3">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>